<commit_message>
Corrected MPN in BOM
</commit_message>
<xml_diff>
--- a/hardware/Self_Watering_POT/BOM.xlsx
+++ b/hardware/Self_Watering_POT/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ProjektySTM\Self_Watering_Pot\hardware\Self_Watering_POT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D05E198-A450-40B2-9072-CD88668E91A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5415AB07-3FE8-48DB-96DA-81E9C5592136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{ED61C653-DEC4-4346-B2F5-304ECAB62126}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED61C653-DEC4-4346-B2F5-304ECAB62126}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -200,15 +200,9 @@
     <t>C2480</t>
   </si>
   <si>
-    <t>C388236</t>
-  </si>
-  <si>
     <t>C141723</t>
   </si>
   <si>
-    <t>C1591</t>
-  </si>
-  <si>
     <t>C7171</t>
   </si>
   <si>
@@ -234,6 +228,12 @@
   </si>
   <si>
     <t>C17513</t>
+  </si>
+  <si>
+    <t>C49678</t>
+  </si>
+  <si>
+    <t>C64982</t>
   </si>
 </sst>
 </file>
@@ -674,7 +674,7 @@
         <v>5</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E2" s="2" t="s">
         <v>6</v>
@@ -691,7 +691,7 @@
         <v>8</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>9</v>
@@ -708,7 +708,7 @@
         <v>11</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>6</v>
@@ -725,7 +725,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>14</v>
@@ -759,7 +759,7 @@
         <v>19</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>51</v>
+        <v>62</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>20</v>
@@ -793,7 +793,7 @@
         <v>24</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>25</v>
@@ -810,7 +810,7 @@
         <v>27</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>28</v>
@@ -827,7 +827,7 @@
         <v>30</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>31</v>
@@ -844,7 +844,7 @@
         <v>33</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>31</v>
@@ -861,7 +861,7 @@
         <v>35</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>31</v>
@@ -878,7 +878,7 @@
         <v>37</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>31</v>
@@ -895,7 +895,7 @@
         <v>39</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E15" s="2" t="s">
         <v>31</v>

</xml_diff>

<commit_message>
Corrected mistakes with PCB board
</commit_message>
<xml_diff>
--- a/hardware/Self_Watering_POT/BOM.xlsx
+++ b/hardware/Self_Watering_POT/BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ProjektySTM\Self_Watering_Pot\hardware\Self_Watering_POT\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5415AB07-3FE8-48DB-96DA-81E9C5592136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FA19C68-A756-4130-82A7-6B9B14F88F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{ED61C653-DEC4-4346-B2F5-304ECAB62126}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{ED61C653-DEC4-4346-B2F5-304ECAB62126}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="66">
   <si>
     <t>Reference</t>
   </si>
@@ -59,9 +59,6 @@
     <t>Footprint</t>
   </si>
   <si>
-    <t>C1,C3</t>
-  </si>
-  <si>
     <t>10uF</t>
   </si>
   <si>
@@ -234,6 +231,18 @@
   </si>
   <si>
     <t>C64982</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>10uF 25V</t>
+  </si>
+  <si>
+    <t>C2158829</t>
   </si>
 </sst>
 </file>
@@ -316,11 +325,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hiperłącze" xfId="1" builtinId="8"/>
@@ -636,7 +646,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C584EC7-7144-4252-8362-4B6877916C07}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.90625" bestFit="1" customWidth="1"/>
@@ -657,289 +667,306 @@
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="2">
-        <v>2</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="A2" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="4">
+        <v>1</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>5</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>62</v>
       </c>
       <c r="B3" s="2">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>61</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="B4" s="2">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B6" s="2">
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>49</v>
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>53</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>62</v>
+        <v>15</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>48</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="B8" s="2">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B9" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="B10" s="2">
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="B11" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="B12" s="2">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B13" s="2">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B14" s="2">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B15" s="2">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B16" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>48</v>
+        <v>38</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>59</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B17" s="2">
         <v>1</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>47</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>45</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B18" s="2">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D17" r:id="rId1" tooltip="C69336" display="https://www.lcsc.com/product-detail/C69336.html?s_z=s_p_STM32F446RET6&amp;spm=wm.fly.bg.0.cbh&amp;lcsc_vid=QAVaXl1fEwdfBlEFElhXBlxWQQJYX1JVEVVaBlNVQQIxVlNeTlFcV1JURlJdUzsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaFA%3D%3D" xr:uid="{1523931D-4F82-4D3E-BDAD-3FCD13B4C737}"/>
-    <hyperlink ref="D16" r:id="rId2" tooltip="C6186" display="https://www.lcsc.com/product-detail/C6186.html?s_z=n_q_p_AMS1117-3.3_SOT223&amp;spm=wm.ssy.bg.0.cbh&amp;lcsc_vid=QAVaXl1fEwdfBlEFElhXBlxWQQJYX1JVEVVaBlNVQQIxVlNeTlFcV1JQR1VeVzsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktfQ1BADxALGw%3D%3D" xr:uid="{937E5B63-63E5-4E28-854F-4337562F8EED}"/>
-    <hyperlink ref="D6" r:id="rId3" tooltip="C83846" display="https://www.lcsc.com/product-detail/C83846.html?s_z=n_q_SMBJ15A&amp;spm=wm.fly.bg.0.cbh&amp;lcsc_vid=QAVaXl1fEwdfBlEFElhXBlxWQQJYX1JVEVVaBlNVQQIxVlNeTlFcV1NVQFdaXjsOAxUeFF5JWBYZEEoKFBINSQcJGk4dAgUUFAk%3D" xr:uid="{AFA5AF85-FC9B-4F6D-9003-82B6FC44B2C7}"/>
+    <hyperlink ref="D18" r:id="rId1" tooltip="C69336" display="https://www.lcsc.com/product-detail/C69336.html?s_z=s_p_STM32F446RET6&amp;spm=wm.fly.bg.0.cbh&amp;lcsc_vid=QAVaXl1fEwdfBlEFElhXBlxWQQJYX1JVEVVaBlNVQQIxVlNeTlFcV1JURlJdUzsOAxUeFF5JWBYZEEoKFBINSQcJGk4eFQsCAgIaFA%3D%3D" xr:uid="{1523931D-4F82-4D3E-BDAD-3FCD13B4C737}"/>
+    <hyperlink ref="D17" r:id="rId2" tooltip="C6186" display="https://www.lcsc.com/product-detail/C6186.html?s_z=n_q_p_AMS1117-3.3_SOT223&amp;spm=wm.ssy.bg.0.cbh&amp;lcsc_vid=QAVaXl1fEwdfBlEFElhXBlxWQQJYX1JVEVVaBlNVQQIxVlNeTlFcV1JQR1VeVzsOAxUeFF5JWBYZEEoKFBINSQcJGk4NBhADEA4cHktfQ1BADxALGw%3D%3D" xr:uid="{937E5B63-63E5-4E28-854F-4337562F8EED}"/>
+    <hyperlink ref="D7" r:id="rId3" tooltip="C83846" display="https://www.lcsc.com/product-detail/C83846.html?s_z=n_q_SMBJ15A&amp;spm=wm.fly.bg.0.cbh&amp;lcsc_vid=QAVaXl1fEwdfBlEFElhXBlxWQQJYX1JVEVVaBlNVQQIxVlNeTlFcV1NVQFdaXjsOAxUeFF5JWBYZEEoKFBINSQcJGk4dAgUUFAk%3D" xr:uid="{AFA5AF85-FC9B-4F6D-9003-82B6FC44B2C7}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>